<commit_message>
Fix Swing bestandsnaam en toevoeging configureerbare swing unit
Co-Authored-By: JoanneNies <131348626+JoanneNies@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/configuratie.xlsx
+++ b/configuratie.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="I:\Github\GGData_tabellenboek\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="I:\Repositories\GGData_tabellenboek\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CC06673E-B887-4E2E-9AFD-ECA14BD84156}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E9AEECD6-7910-4D82-9BDE-E9B906BF5A69}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4680" yWindow="4680" windowWidth="38700" windowHeight="15345" tabRatio="731" xr2:uid="{ECC980AC-D294-4808-BCB8-F5A87956E45F}"/>
+    <workbookView xWindow="0" yWindow="315" windowWidth="28905" windowHeight="15240" tabRatio="731" xr2:uid="{ECC980AC-D294-4808-BCB8-F5A87956E45F}"/>
   </bookViews>
   <sheets>
     <sheet name="algemeen" sheetId="5" r:id="rId1"/>
@@ -51,7 +51,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="277" uniqueCount="212">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="279" uniqueCount="214">
   <si>
     <t>naam_dataset</t>
   </si>
@@ -687,6 +687,12 @@
   </si>
   <si>
     <t>swing_afkapwaarde</t>
+  </si>
+  <si>
+    <t>swing_unit</t>
+  </si>
+  <si>
+    <t>p</t>
   </si>
 </sst>
 </file>
@@ -1057,7 +1063,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CB9555E0-3443-4710-AD14-3A977E907E6B}">
-  <dimension ref="A1:U2"/>
+  <dimension ref="A1:V2"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="13.42578125" customWidth="1"/>
@@ -1072,7 +1078,7 @@
     <col min="18" max="18" width="9.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>55</v>
       </c>
@@ -1136,8 +1142,11 @@
       <c r="U1" t="s">
         <v>211</v>
       </c>
-    </row>
-    <row r="2" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="V1" t="s">
+        <v>212</v>
+      </c>
+    </row>
+    <row r="2" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>10</v>
       </c>
@@ -1200,6 +1209,9 @@
       </c>
       <c r="U2">
         <v>-99996</v>
+      </c>
+      <c r="V2" t="s">
+        <v>213</v>
       </c>
     </row>
   </sheetData>

</xml_diff>